<commit_message>
Regenerate output templates; reference results for the fake school
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B1DqxLw2MywB8g5N8E14F5
</commit_message>
<xml_diff>
--- a/data/Output_Template_Thong_Ke_V8.xlsx
+++ b/data/Output_Template_Thong_Ke_V8.xlsx
@@ -1150,10 +1150,10 @@
       <c r="H16" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I16" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n">
         <v>2</v>
@@ -1167,7 +1167,7 @@
       <c r="Q16" s="2" t="n"/>
       <c r="R16" s="2" t="n"/>
       <c r="S16" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" ht="25" customHeight="1">
@@ -1240,10 +1240,10 @@
       <c r="H18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I18" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J18" s="2" t="n"/>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n">
         <v>2</v>
@@ -1257,7 +1257,7 @@
       <c r="Q18" s="2" t="n"/>
       <c r="R18" s="2" t="n"/>
       <c r="S18" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" ht="25" customHeight="1">
@@ -1337,7 +1337,9 @@
       <c r="I20" s="2" t="n"/>
       <c r="J20" s="2" t="n"/>
       <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
+      <c r="L20" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="M20" s="2" t="n"/>
       <c r="N20" s="2" t="n"/>
       <c r="O20" s="2" t="n"/>
@@ -1345,7 +1347,7 @@
       <c r="Q20" s="2" t="n"/>
       <c r="R20" s="2" t="n"/>
       <c r="S20" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" ht="25" customHeight="1">
@@ -1470,7 +1472,9 @@
       <c r="I23" s="2" t="n"/>
       <c r="J23" s="2" t="n"/>
       <c r="K23" s="2" t="n"/>
-      <c r="L23" s="2" t="n"/>
+      <c r="L23" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="M23" s="2" t="n"/>
       <c r="N23" s="2" t="n"/>
       <c r="O23" s="2" t="n"/>
@@ -1478,7 +1482,7 @@
       <c r="Q23" s="2" t="n"/>
       <c r="R23" s="2" t="n"/>
       <c r="S23" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24" ht="25" customHeight="1">
@@ -1806,7 +1810,7 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="n"/>
@@ -1814,24 +1818,18 @@
       <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="K31" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="L31" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="K31" s="2" t="n"/>
+      <c r="L31" s="2" t="n"/>
       <c r="M31" s="2" t="n"/>
       <c r="N31" s="2" t="n"/>
       <c r="O31" s="2" t="n"/>
       <c r="P31" s="2" t="n"/>
-      <c r="Q31" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="Q31" s="2" t="n"/>
       <c r="R31" s="2" t="n"/>
       <c r="S31" s="2" t="n">
         <v>23</v>
@@ -1849,7 +1847,7 @@
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="n"/>
@@ -1857,24 +1855,20 @@
       <c r="G32" s="2" t="n"/>
       <c r="H32" s="2" t="n"/>
       <c r="I32" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K32" s="2" t="n"/>
+      <c r="L32" s="2" t="n">
         <v>6</v>
-      </c>
-      <c r="J32" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="K32" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="L32" s="2" t="n">
-        <v>2</v>
       </c>
       <c r="M32" s="2" t="n"/>
       <c r="N32" s="2" t="n"/>
       <c r="O32" s="2" t="n"/>
       <c r="P32" s="2" t="n"/>
-      <c r="Q32" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q32" s="2" t="n"/>
       <c r="R32" s="2" t="n"/>
       <c r="S32" s="2" t="n">
         <v>23</v>
@@ -1891,25 +1885,23 @@
           <t>Bộ Môn 3</t>
         </is>
       </c>
-      <c r="C33" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="C33" s="2" t="n"/>
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="n"/>
       <c r="H33" s="2" t="n"/>
       <c r="I33" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M33" s="2" t="n"/>
       <c r="N33" s="2" t="n"/>
@@ -1942,24 +1934,18 @@
         <v>6</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="L34" s="2" t="n">
-        <v>4</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="L34" s="2" t="n"/>
       <c r="M34" s="2" t="n"/>
       <c r="N34" s="2" t="n"/>
       <c r="O34" s="2" t="n"/>
       <c r="P34" s="2" t="n"/>
-      <c r="Q34" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="R34" s="2" t="n">
-        <v>6</v>
-      </c>
+      <c r="Q34" s="2" t="n"/>
+      <c r="R34" s="2" t="n"/>
       <c r="S34" s="2" t="n">
         <v>23</v>
       </c>
@@ -1976,29 +1962,33 @@
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="n"/>
       <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J35" s="2" t="n"/>
-      <c r="K35" s="2" t="n"/>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K35" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="L35" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M35" s="2" t="n"/>
       <c r="N35" s="2" t="n"/>
       <c r="O35" s="2" t="n"/>
       <c r="P35" s="2" t="n"/>
       <c r="Q35" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R35" s="2" t="n"/>
+        <v>6</v>
+      </c>
+      <c r="R35" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="S35" s="2" t="n">
         <v>19</v>
       </c>
@@ -2160,12 +2150,12 @@
       <c r="N40" s="2" t="n"/>
       <c r="O40" s="2" t="n"/>
       <c r="P40" s="2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="Q40" s="2" t="n"/>
       <c r="R40" s="2" t="n"/>
       <c r="S40" s="2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="41" ht="25" customHeight="1">
@@ -2193,12 +2183,12 @@
       <c r="N41" s="2" t="n"/>
       <c r="O41" s="2" t="n"/>
       <c r="P41" s="2" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="Q41" s="2" t="n"/>
       <c r="R41" s="2" t="n"/>
       <c r="S41" s="2" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="42" ht="25" customHeight="1">
@@ -2226,12 +2216,12 @@
       <c r="N42" s="2" t="n"/>
       <c r="O42" s="2" t="n"/>
       <c r="P42" s="2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="Q42" s="2" t="n"/>
       <c r="R42" s="2" t="n"/>
       <c r="S42" s="2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="43" ht="25" customHeight="1">

</xml_diff>

<commit_message>
Regenerate statistics template with highlighted overtime rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B1DqxLw2MywB8g5N8E14F5
</commit_message>
<xml_diff>
--- a/data/Output_Template_Thong_Ke_V8.xlsx
+++ b/data/Output_Template_Thong_Ke_V8.xlsx
@@ -35,12 +35,18 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -61,13 +67,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -434,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S47"/>
+  <dimension ref="A1:S49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20.3" customWidth="1" min="1" max="1"/>
@@ -1799,560 +1811,560 @@
       </c>
     </row>
     <row r="31" ht="25" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Giáo viên BM 1</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Bộ Môn 1</t>
         </is>
       </c>
-      <c r="C31" s="2" t="n">
+      <c r="C31" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
-      <c r="G31" s="2" t="n"/>
-      <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="n">
+      <c r="D31" s="3" t="n"/>
+      <c r="E31" s="3" t="n"/>
+      <c r="F31" s="3" t="n"/>
+      <c r="G31" s="3" t="n"/>
+      <c r="H31" s="3" t="n"/>
+      <c r="I31" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="J31" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K31" s="2" t="n"/>
-      <c r="L31" s="2" t="n"/>
-      <c r="M31" s="2" t="n"/>
-      <c r="N31" s="2" t="n"/>
-      <c r="O31" s="2" t="n"/>
-      <c r="P31" s="2" t="n"/>
-      <c r="Q31" s="2" t="n"/>
-      <c r="R31" s="2" t="n"/>
-      <c r="S31" s="2" t="n">
+      <c r="J31" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K31" s="3" t="n"/>
+      <c r="L31" s="3" t="n"/>
+      <c r="M31" s="3" t="n"/>
+      <c r="N31" s="3" t="n"/>
+      <c r="O31" s="3" t="n"/>
+      <c r="P31" s="3" t="n"/>
+      <c r="Q31" s="3" t="n"/>
+      <c r="R31" s="3" t="n"/>
+      <c r="S31" s="3" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="32" ht="25" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Giáo viên BM 2</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Bộ Môn 2</t>
         </is>
       </c>
-      <c r="C32" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
-      <c r="G32" s="2" t="n"/>
-      <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="n">
+      <c r="C32" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" s="3" t="n"/>
+      <c r="E32" s="3" t="n"/>
+      <c r="F32" s="3" t="n"/>
+      <c r="G32" s="3" t="n"/>
+      <c r="H32" s="3" t="n"/>
+      <c r="I32" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="J32" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K32" s="2" t="n"/>
-      <c r="L32" s="2" t="n">
+      <c r="J32" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K32" s="3" t="n"/>
+      <c r="L32" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="M32" s="2" t="n"/>
-      <c r="N32" s="2" t="n"/>
-      <c r="O32" s="2" t="n"/>
-      <c r="P32" s="2" t="n"/>
-      <c r="Q32" s="2" t="n"/>
-      <c r="R32" s="2" t="n"/>
-      <c r="S32" s="2" t="n">
+      <c r="M32" s="3" t="n"/>
+      <c r="N32" s="3" t="n"/>
+      <c r="O32" s="3" t="n"/>
+      <c r="P32" s="3" t="n"/>
+      <c r="Q32" s="3" t="n"/>
+      <c r="R32" s="3" t="n"/>
+      <c r="S32" s="3" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="33" ht="25" customHeight="1">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Giáo viên BM 3</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Bộ Môn 3</t>
         </is>
       </c>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
-      <c r="G33" s="2" t="n"/>
-      <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n">
+      <c r="C33" s="3" t="n"/>
+      <c r="D33" s="3" t="n"/>
+      <c r="E33" s="3" t="n"/>
+      <c r="F33" s="3" t="n"/>
+      <c r="G33" s="3" t="n"/>
+      <c r="H33" s="3" t="n"/>
+      <c r="I33" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="J33" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K33" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="L33" s="2" t="n">
+      <c r="J33" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K33" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="L33" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="M33" s="2" t="n"/>
-      <c r="N33" s="2" t="n"/>
-      <c r="O33" s="2" t="n"/>
-      <c r="P33" s="2" t="n"/>
-      <c r="Q33" s="2" t="n"/>
-      <c r="R33" s="2" t="n"/>
-      <c r="S33" s="2" t="n">
+      <c r="M33" s="3" t="n"/>
+      <c r="N33" s="3" t="n"/>
+      <c r="O33" s="3" t="n"/>
+      <c r="P33" s="3" t="n"/>
+      <c r="Q33" s="3" t="n"/>
+      <c r="R33" s="3" t="n"/>
+      <c r="S33" s="3" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="34" ht="25" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>Giáo viên BM 4</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Bộ Môn 4</t>
         </is>
       </c>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n">
+      <c r="C34" s="3" t="n"/>
+      <c r="D34" s="3" t="n"/>
+      <c r="E34" s="3" t="n"/>
+      <c r="F34" s="3" t="n"/>
+      <c r="G34" s="3" t="n"/>
+      <c r="H34" s="3" t="n"/>
+      <c r="I34" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="J34" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K34" s="2" t="n">
+      <c r="J34" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K34" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="L34" s="2" t="n"/>
-      <c r="M34" s="2" t="n"/>
-      <c r="N34" s="2" t="n"/>
-      <c r="O34" s="2" t="n"/>
-      <c r="P34" s="2" t="n"/>
-      <c r="Q34" s="2" t="n"/>
-      <c r="R34" s="2" t="n"/>
-      <c r="S34" s="2" t="n">
+      <c r="L34" s="3" t="n"/>
+      <c r="M34" s="3" t="n"/>
+      <c r="N34" s="3" t="n"/>
+      <c r="O34" s="3" t="n"/>
+      <c r="P34" s="3" t="n"/>
+      <c r="Q34" s="3" t="n"/>
+      <c r="R34" s="3" t="n"/>
+      <c r="S34" s="3" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="35" ht="25" customHeight="1">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Giáo viên BM 5</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Bộ Môn 5</t>
         </is>
       </c>
-      <c r="C35" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="n"/>
-      <c r="G35" s="2" t="n"/>
-      <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="n"/>
-      <c r="J35" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K35" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="L35" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M35" s="2" t="n"/>
-      <c r="N35" s="2" t="n"/>
-      <c r="O35" s="2" t="n"/>
-      <c r="P35" s="2" t="n"/>
-      <c r="Q35" s="2" t="n">
+      <c r="C35" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" s="3" t="n"/>
+      <c r="E35" s="3" t="n"/>
+      <c r="F35" s="3" t="n"/>
+      <c r="G35" s="3" t="n"/>
+      <c r="H35" s="3" t="n"/>
+      <c r="I35" s="3" t="n"/>
+      <c r="J35" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K35" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="L35" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M35" s="3" t="n"/>
+      <c r="N35" s="3" t="n"/>
+      <c r="O35" s="3" t="n"/>
+      <c r="P35" s="3" t="n"/>
+      <c r="Q35" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="R35" s="2" t="n">
+      <c r="R35" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="S35" s="2" t="n">
+      <c r="S35" s="3" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="36" ht="25" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>Giáo viên TA 1</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Tiếng Anh 1</t>
         </is>
       </c>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
-      <c r="J36" s="2" t="n"/>
-      <c r="K36" s="2" t="n"/>
-      <c r="L36" s="2" t="n"/>
-      <c r="M36" s="2" t="n"/>
-      <c r="N36" s="2" t="n">
+      <c r="C36" s="3" t="n"/>
+      <c r="D36" s="3" t="n"/>
+      <c r="E36" s="3" t="n"/>
+      <c r="F36" s="3" t="n"/>
+      <c r="G36" s="3" t="n"/>
+      <c r="H36" s="3" t="n"/>
+      <c r="I36" s="3" t="n"/>
+      <c r="J36" s="3" t="n"/>
+      <c r="K36" s="3" t="n"/>
+      <c r="L36" s="3" t="n"/>
+      <c r="M36" s="3" t="n"/>
+      <c r="N36" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="O36" s="2" t="n"/>
-      <c r="P36" s="2" t="n"/>
-      <c r="Q36" s="2" t="n"/>
-      <c r="R36" s="2" t="n"/>
-      <c r="S36" s="2" t="n">
+      <c r="O36" s="3" t="n"/>
+      <c r="P36" s="3" t="n"/>
+      <c r="Q36" s="3" t="n"/>
+      <c r="R36" s="3" t="n"/>
+      <c r="S36" s="3" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="37" ht="25" customHeight="1">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>Giáo viên TA 2</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>Tiếng Anh 2</t>
         </is>
       </c>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
-      <c r="J37" s="2" t="n"/>
-      <c r="K37" s="2" t="n"/>
-      <c r="L37" s="2" t="n"/>
-      <c r="M37" s="2" t="n"/>
-      <c r="N37" s="2" t="n">
+      <c r="C37" s="3" t="n"/>
+      <c r="D37" s="3" t="n"/>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="n"/>
+      <c r="G37" s="3" t="n"/>
+      <c r="H37" s="3" t="n"/>
+      <c r="I37" s="3" t="n"/>
+      <c r="J37" s="3" t="n"/>
+      <c r="K37" s="3" t="n"/>
+      <c r="L37" s="3" t="n"/>
+      <c r="M37" s="3" t="n"/>
+      <c r="N37" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="O37" s="2" t="n"/>
-      <c r="P37" s="2" t="n"/>
-      <c r="Q37" s="2" t="n"/>
-      <c r="R37" s="2" t="n"/>
-      <c r="S37" s="2" t="n">
+      <c r="O37" s="3" t="n"/>
+      <c r="P37" s="3" t="n"/>
+      <c r="Q37" s="3" t="n"/>
+      <c r="R37" s="3" t="n"/>
+      <c r="S37" s="3" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="38" ht="25" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>Giáo viên TA 3</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>Tiếng Anh 3</t>
         </is>
       </c>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
-      <c r="G38" s="2" t="n"/>
-      <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="n"/>
-      <c r="J38" s="2" t="n"/>
-      <c r="K38" s="2" t="n"/>
-      <c r="L38" s="2" t="n"/>
-      <c r="M38" s="2" t="n"/>
-      <c r="N38" s="2" t="n">
+      <c r="C38" s="3" t="n"/>
+      <c r="D38" s="3" t="n"/>
+      <c r="E38" s="3" t="n"/>
+      <c r="F38" s="3" t="n"/>
+      <c r="G38" s="3" t="n"/>
+      <c r="H38" s="3" t="n"/>
+      <c r="I38" s="3" t="n"/>
+      <c r="J38" s="3" t="n"/>
+      <c r="K38" s="3" t="n"/>
+      <c r="L38" s="3" t="n"/>
+      <c r="M38" s="3" t="n"/>
+      <c r="N38" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="O38" s="2" t="n"/>
-      <c r="P38" s="2" t="n"/>
-      <c r="Q38" s="2" t="n"/>
-      <c r="R38" s="2" t="n"/>
-      <c r="S38" s="2" t="n">
+      <c r="O38" s="3" t="n"/>
+      <c r="P38" s="3" t="n"/>
+      <c r="Q38" s="3" t="n"/>
+      <c r="R38" s="3" t="n"/>
+      <c r="S38" s="3" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="39" ht="25" customHeight="1">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>Giáo viên TA 4</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Tiếng Anh 4</t>
         </is>
       </c>
-      <c r="C39" s="2" t="n"/>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="2" t="n"/>
-      <c r="G39" s="2" t="n"/>
-      <c r="H39" s="2" t="n"/>
-      <c r="I39" s="2" t="n"/>
-      <c r="J39" s="2" t="n"/>
-      <c r="K39" s="2" t="n"/>
-      <c r="L39" s="2" t="n"/>
-      <c r="M39" s="2" t="n"/>
-      <c r="N39" s="2" t="n">
+      <c r="C39" s="3" t="n"/>
+      <c r="D39" s="3" t="n"/>
+      <c r="E39" s="3" t="n"/>
+      <c r="F39" s="3" t="n"/>
+      <c r="G39" s="3" t="n"/>
+      <c r="H39" s="3" t="n"/>
+      <c r="I39" s="3" t="n"/>
+      <c r="J39" s="3" t="n"/>
+      <c r="K39" s="3" t="n"/>
+      <c r="L39" s="3" t="n"/>
+      <c r="M39" s="3" t="n"/>
+      <c r="N39" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="O39" s="2" t="n"/>
-      <c r="P39" s="2" t="n"/>
-      <c r="Q39" s="2" t="n"/>
-      <c r="R39" s="2" t="n"/>
-      <c r="S39" s="2" t="n">
+      <c r="O39" s="3" t="n"/>
+      <c r="P39" s="3" t="n"/>
+      <c r="Q39" s="3" t="n"/>
+      <c r="R39" s="3" t="n"/>
+      <c r="S39" s="3" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="40" ht="25" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>Giáo viên TD 1</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>Thể Dục 1</t>
         </is>
       </c>
-      <c r="C40" s="2" t="n"/>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="2" t="n"/>
-      <c r="G40" s="2" t="n"/>
-      <c r="H40" s="2" t="n"/>
-      <c r="I40" s="2" t="n"/>
-      <c r="J40" s="2" t="n"/>
-      <c r="K40" s="2" t="n"/>
-      <c r="L40" s="2" t="n"/>
-      <c r="M40" s="2" t="n"/>
-      <c r="N40" s="2" t="n"/>
-      <c r="O40" s="2" t="n"/>
-      <c r="P40" s="2" t="n">
+      <c r="C40" s="3" t="n"/>
+      <c r="D40" s="3" t="n"/>
+      <c r="E40" s="3" t="n"/>
+      <c r="F40" s="3" t="n"/>
+      <c r="G40" s="3" t="n"/>
+      <c r="H40" s="3" t="n"/>
+      <c r="I40" s="3" t="n"/>
+      <c r="J40" s="3" t="n"/>
+      <c r="K40" s="3" t="n"/>
+      <c r="L40" s="3" t="n"/>
+      <c r="M40" s="3" t="n"/>
+      <c r="N40" s="3" t="n"/>
+      <c r="O40" s="3" t="n"/>
+      <c r="P40" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="Q40" s="2" t="n"/>
-      <c r="R40" s="2" t="n"/>
-      <c r="S40" s="2" t="n">
+      <c r="Q40" s="3" t="n"/>
+      <c r="R40" s="3" t="n"/>
+      <c r="S40" s="3" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="41" ht="25" customHeight="1">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>Giáo viên TD 2</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>Thể Dục 2</t>
         </is>
       </c>
-      <c r="C41" s="2" t="n"/>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="2" t="n"/>
-      <c r="G41" s="2" t="n"/>
-      <c r="H41" s="2" t="n"/>
-      <c r="I41" s="2" t="n"/>
-      <c r="J41" s="2" t="n"/>
-      <c r="K41" s="2" t="n"/>
-      <c r="L41" s="2" t="n"/>
-      <c r="M41" s="2" t="n"/>
-      <c r="N41" s="2" t="n"/>
-      <c r="O41" s="2" t="n"/>
-      <c r="P41" s="2" t="n">
+      <c r="C41" s="3" t="n"/>
+      <c r="D41" s="3" t="n"/>
+      <c r="E41" s="3" t="n"/>
+      <c r="F41" s="3" t="n"/>
+      <c r="G41" s="3" t="n"/>
+      <c r="H41" s="3" t="n"/>
+      <c r="I41" s="3" t="n"/>
+      <c r="J41" s="3" t="n"/>
+      <c r="K41" s="3" t="n"/>
+      <c r="L41" s="3" t="n"/>
+      <c r="M41" s="3" t="n"/>
+      <c r="N41" s="3" t="n"/>
+      <c r="O41" s="3" t="n"/>
+      <c r="P41" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="Q41" s="2" t="n"/>
-      <c r="R41" s="2" t="n"/>
-      <c r="S41" s="2" t="n">
+      <c r="Q41" s="3" t="n"/>
+      <c r="R41" s="3" t="n"/>
+      <c r="S41" s="3" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="42" ht="25" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>Giáo viên TD 3</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>Thể Dục 3</t>
         </is>
       </c>
-      <c r="C42" s="2" t="n"/>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="n"/>
-      <c r="G42" s="2" t="n"/>
-      <c r="H42" s="2" t="n"/>
-      <c r="I42" s="2" t="n"/>
-      <c r="J42" s="2" t="n"/>
-      <c r="K42" s="2" t="n"/>
-      <c r="L42" s="2" t="n"/>
-      <c r="M42" s="2" t="n"/>
-      <c r="N42" s="2" t="n"/>
-      <c r="O42" s="2" t="n"/>
-      <c r="P42" s="2" t="n">
+      <c r="C42" s="3" t="n"/>
+      <c r="D42" s="3" t="n"/>
+      <c r="E42" s="3" t="n"/>
+      <c r="F42" s="3" t="n"/>
+      <c r="G42" s="3" t="n"/>
+      <c r="H42" s="3" t="n"/>
+      <c r="I42" s="3" t="n"/>
+      <c r="J42" s="3" t="n"/>
+      <c r="K42" s="3" t="n"/>
+      <c r="L42" s="3" t="n"/>
+      <c r="M42" s="3" t="n"/>
+      <c r="N42" s="3" t="n"/>
+      <c r="O42" s="3" t="n"/>
+      <c r="P42" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="Q42" s="2" t="n"/>
-      <c r="R42" s="2" t="n"/>
-      <c r="S42" s="2" t="n">
+      <c r="Q42" s="3" t="n"/>
+      <c r="R42" s="3" t="n"/>
+      <c r="S42" s="3" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="43" ht="25" customHeight="1">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>Giáo viên ÂN 1</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>Âm Nhạc 1</t>
         </is>
       </c>
-      <c r="C43" s="2" t="n"/>
-      <c r="D43" s="2" t="n"/>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="n"/>
-      <c r="G43" s="2" t="n"/>
-      <c r="H43" s="2" t="n"/>
-      <c r="I43" s="2" t="n"/>
-      <c r="J43" s="2" t="n"/>
-      <c r="K43" s="2" t="n"/>
-      <c r="L43" s="2" t="n"/>
-      <c r="M43" s="2" t="n"/>
-      <c r="N43" s="2" t="n"/>
-      <c r="O43" s="2" t="n"/>
-      <c r="P43" s="2" t="n"/>
-      <c r="Q43" s="2" t="n">
+      <c r="C43" s="3" t="n"/>
+      <c r="D43" s="3" t="n"/>
+      <c r="E43" s="3" t="n"/>
+      <c r="F43" s="3" t="n"/>
+      <c r="G43" s="3" t="n"/>
+      <c r="H43" s="3" t="n"/>
+      <c r="I43" s="3" t="n"/>
+      <c r="J43" s="3" t="n"/>
+      <c r="K43" s="3" t="n"/>
+      <c r="L43" s="3" t="n"/>
+      <c r="M43" s="3" t="n"/>
+      <c r="N43" s="3" t="n"/>
+      <c r="O43" s="3" t="n"/>
+      <c r="P43" s="3" t="n"/>
+      <c r="Q43" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="R43" s="2" t="n"/>
-      <c r="S43" s="2" t="n">
+      <c r="R43" s="3" t="n"/>
+      <c r="S43" s="3" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="44" ht="25" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>Giáo viên MT 1</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>Mỹ Thuật 1</t>
         </is>
       </c>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
-      <c r="G44" s="2" t="n"/>
-      <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="n"/>
-      <c r="J44" s="2" t="n"/>
-      <c r="K44" s="2" t="n"/>
-      <c r="L44" s="2" t="n"/>
-      <c r="M44" s="2" t="n"/>
-      <c r="N44" s="2" t="n"/>
-      <c r="O44" s="2" t="n"/>
-      <c r="P44" s="2" t="n"/>
-      <c r="Q44" s="2" t="n"/>
-      <c r="R44" s="2" t="n">
+      <c r="C44" s="3" t="n"/>
+      <c r="D44" s="3" t="n"/>
+      <c r="E44" s="3" t="n"/>
+      <c r="F44" s="3" t="n"/>
+      <c r="G44" s="3" t="n"/>
+      <c r="H44" s="3" t="n"/>
+      <c r="I44" s="3" t="n"/>
+      <c r="J44" s="3" t="n"/>
+      <c r="K44" s="3" t="n"/>
+      <c r="L44" s="3" t="n"/>
+      <c r="M44" s="3" t="n"/>
+      <c r="N44" s="3" t="n"/>
+      <c r="O44" s="3" t="n"/>
+      <c r="P44" s="3" t="n"/>
+      <c r="Q44" s="3" t="n"/>
+      <c r="R44" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="S44" s="2" t="n">
+      <c r="S44" s="3" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="45" ht="25" customHeight="1">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>Giáo viên TH 1</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>Tin Học 1</t>
         </is>
       </c>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
-      <c r="G45" s="2" t="n"/>
-      <c r="H45" s="2" t="n"/>
-      <c r="I45" s="2" t="n"/>
-      <c r="J45" s="2" t="n"/>
-      <c r="K45" s="2" t="n"/>
-      <c r="L45" s="2" t="n"/>
-      <c r="M45" s="2" t="n"/>
-      <c r="N45" s="2" t="n"/>
-      <c r="O45" s="2" t="n">
+      <c r="C45" s="3" t="n"/>
+      <c r="D45" s="3" t="n"/>
+      <c r="E45" s="3" t="n"/>
+      <c r="F45" s="3" t="n"/>
+      <c r="G45" s="3" t="n"/>
+      <c r="H45" s="3" t="n"/>
+      <c r="I45" s="3" t="n"/>
+      <c r="J45" s="3" t="n"/>
+      <c r="K45" s="3" t="n"/>
+      <c r="L45" s="3" t="n"/>
+      <c r="M45" s="3" t="n"/>
+      <c r="N45" s="3" t="n"/>
+      <c r="O45" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="P45" s="2" t="n"/>
-      <c r="Q45" s="2" t="n"/>
-      <c r="R45" s="2" t="n"/>
-      <c r="S45" s="2" t="n">
+      <c r="P45" s="3" t="n"/>
+      <c r="Q45" s="3" t="n"/>
+      <c r="R45" s="3" t="n"/>
+      <c r="S45" s="3" t="n">
         <v>17</v>
       </c>
     </row>
     <row r="46" ht="25" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>Giáo viên QL 1</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>Quản Lý 1</t>
         </is>
       </c>
-      <c r="C46" s="2" t="n"/>
-      <c r="D46" s="2" t="n"/>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="2" t="n"/>
-      <c r="G46" s="2" t="n"/>
-      <c r="H46" s="2" t="n"/>
-      <c r="I46" s="2" t="n"/>
-      <c r="J46" s="2" t="n">
+      <c r="C46" s="3" t="n"/>
+      <c r="D46" s="3" t="n"/>
+      <c r="E46" s="3" t="n"/>
+      <c r="F46" s="3" t="n"/>
+      <c r="G46" s="3" t="n"/>
+      <c r="H46" s="3" t="n"/>
+      <c r="I46" s="3" t="n"/>
+      <c r="J46" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="K46" s="2" t="n"/>
-      <c r="L46" s="2" t="n"/>
-      <c r="M46" s="2" t="n"/>
-      <c r="N46" s="2" t="n"/>
-      <c r="O46" s="2" t="n"/>
-      <c r="P46" s="2" t="n"/>
-      <c r="Q46" s="2" t="n"/>
-      <c r="R46" s="2" t="n"/>
-      <c r="S46" s="2" t="n">
+      <c r="K46" s="3" t="n"/>
+      <c r="L46" s="3" t="n"/>
+      <c r="M46" s="3" t="n"/>
+      <c r="N46" s="3" t="n"/>
+      <c r="O46" s="3" t="n"/>
+      <c r="P46" s="3" t="n"/>
+      <c r="Q46" s="3" t="n"/>
+      <c r="R46" s="3" t="n"/>
+      <c r="S46" s="3" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2413,6 +2425,15 @@
       </c>
       <c r="S47" s="1" t="n">
         <v>928</v>
+      </c>
+    </row>
+    <row r="48"/>
+    <row r="49" ht="25" customHeight="1">
+      <c r="A49" s="2" t="n"/>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Dạy bù (vượt định mức): 29 người, 52 tiết</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Output templates without cell comments
Regenerated with tools/mau_dau_ra.py (fake-name school, code
428A-3655-C110 unchanged): the statistics template now has the Môn Dạy Bù
column instead of comments in the orange cells.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B1DqxLw2MywB8g5N8E14F5
</commit_message>
<xml_diff>
--- a/data/Output_Template_Thong_Ke_V8.xlsx
+++ b/data/Output_Template_Thong_Ke_V8.xlsx
@@ -173,211 +173,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>TKB</author>
-  </authors>
-  <commentList>
-    <comment ref="C2" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 2 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="C3" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 2 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="C4" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 2 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="C5" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 2 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="C6" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 2 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="C7" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 2 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="M8" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 2 tiết TV tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="M9" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 2 tiết TV tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="M10" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 2 tiết TV tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="M11" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 2 tiết TV tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="M12" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 2 tiết TV tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="M13" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 2 tiết TV tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="J14" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Kỹ năng sống</t>
-      </text>
-    </comment>
-    <comment ref="J15" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Kỹ năng sống</t>
-      </text>
-    </comment>
-    <comment ref="J16" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Kỹ năng sống</t>
-      </text>
-    </comment>
-    <comment ref="J17" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Kỹ năng sống</t>
-      </text>
-    </comment>
-    <comment ref="J18" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Kỹ năng sống</t>
-      </text>
-    </comment>
-    <comment ref="J19" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Kỹ năng sống</t>
-      </text>
-    </comment>
-    <comment ref="C20" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="L20" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Toán tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="C21" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="L21" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Toán tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="C22" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="L22" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Toán tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="C23" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="L23" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Toán tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="C24" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="L24" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Toán tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="C25" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="L25" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Toán tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="C26" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="L26" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Toán tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="C27" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="L27" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Toán tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="C28" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="L28" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Toán tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="C29" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-    <comment ref="L29" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 1 tiết Toán tăng cường</t>
-      </text>
-    </comment>
-    <comment ref="C30" authorId="0" shapeId="0">
-      <text>
-        <t>Dạy bù 2 tiết Tiếng Việt</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -669,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V51"/>
+  <dimension ref="A1:W51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20.3" customWidth="1" min="1" max="1"/>
@@ -693,7 +488,8 @@
     <col width="13" customWidth="1" min="19" max="19"/>
     <col width="16.6" customWidth="1" min="20" max="20"/>
     <col width="14.2" customWidth="1" min="21" max="21"/>
-    <col width="14.2" customWidth="1" min="22" max="22"/>
+    <col width="39.7" customWidth="1" min="22" max="22"/>
+    <col width="14.2" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -803,6 +599,11 @@
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Môn Dạy Bù</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Số Tiết Dư</t>
         </is>
@@ -852,7 +653,12 @@
       <c r="U2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V2" s="2" t="n"/>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 2</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="n"/>
     </row>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -898,7 +704,12 @@
       <c r="U3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V3" s="2" t="n"/>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 2</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="n"/>
     </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -944,7 +755,12 @@
       <c r="U4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V4" s="2" t="n"/>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 2</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="n"/>
     </row>
     <row r="5" ht="25" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -990,7 +806,12 @@
       <c r="U5" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V5" s="2" t="n"/>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 2</t>
+        </is>
+      </c>
+      <c r="W5" s="2" t="n"/>
     </row>
     <row r="6" ht="25" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -1036,7 +857,12 @@
       <c r="U6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V6" s="2" t="n"/>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 2</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="n"/>
     </row>
     <row r="7" ht="25" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -1082,7 +908,12 @@
       <c r="U7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V7" s="2" t="n"/>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 2</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="n"/>
     </row>
     <row r="8" ht="25" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1130,7 +961,12 @@
       <c r="U8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V8" s="2" t="n"/>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>TV tăng cường 2</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="n"/>
     </row>
     <row r="9" ht="25" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -1178,7 +1014,12 @@
       <c r="U9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V9" s="2" t="n"/>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>TV tăng cường 2</t>
+        </is>
+      </c>
+      <c r="W9" s="2" t="n"/>
     </row>
     <row r="10" ht="25" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1226,7 +1067,12 @@
       <c r="U10" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V10" s="2" t="n"/>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>TV tăng cường 2</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="n"/>
     </row>
     <row r="11" ht="25" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -1274,7 +1120,12 @@
       <c r="U11" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V11" s="2" t="n"/>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>TV tăng cường 2</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="n"/>
     </row>
     <row r="12" ht="25" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1322,7 +1173,12 @@
       <c r="U12" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V12" s="2" t="n"/>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>TV tăng cường 2</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="n"/>
     </row>
     <row r="13" ht="25" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -1370,7 +1226,12 @@
       <c r="U13" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V13" s="2" t="n"/>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>TV tăng cường 2</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="n"/>
     </row>
     <row r="14" ht="25" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1422,7 +1283,12 @@
       <c r="U14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V14" s="2" t="n"/>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>Kỹ năng sống 1</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="n"/>
     </row>
     <row r="15" ht="25" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -1474,7 +1340,12 @@
       <c r="U15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V15" s="2" t="n"/>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>Kỹ năng sống 1</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="n"/>
     </row>
     <row r="16" ht="25" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -1526,7 +1397,12 @@
       <c r="U16" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V16" s="2" t="n"/>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>Kỹ năng sống 1</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="n"/>
     </row>
     <row r="17" ht="25" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -1578,7 +1454,12 @@
       <c r="U17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V17" s="2" t="n"/>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>Kỹ năng sống 1</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="n"/>
     </row>
     <row r="18" ht="25" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -1630,7 +1511,12 @@
       <c r="U18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V18" s="2" t="n"/>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t>Kỹ năng sống 1</t>
+        </is>
+      </c>
+      <c r="W18" s="2" t="n"/>
     </row>
     <row r="19" ht="25" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -1682,7 +1568,12 @@
       <c r="U19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V19" s="2" t="n"/>
+      <c r="V19" s="2" t="inlineStr">
+        <is>
+          <t>Kỹ năng sống 1</t>
+        </is>
+      </c>
+      <c r="W19" s="2" t="n"/>
     </row>
     <row r="20" ht="25" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -1734,7 +1625,12 @@
       <c r="U20" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V20" s="2" t="n"/>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 1, Toán tăng cường 1</t>
+        </is>
+      </c>
+      <c r="W20" s="2" t="n"/>
     </row>
     <row r="21" ht="25" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -1786,7 +1682,12 @@
       <c r="U21" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V21" s="2" t="n"/>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 1, Toán tăng cường 1</t>
+        </is>
+      </c>
+      <c r="W21" s="2" t="n"/>
     </row>
     <row r="22" ht="25" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -1838,7 +1739,12 @@
       <c r="U22" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V22" s="2" t="n"/>
+      <c r="V22" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 1, Toán tăng cường 1</t>
+        </is>
+      </c>
+      <c r="W22" s="2" t="n"/>
     </row>
     <row r="23" ht="25" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -1890,7 +1796,12 @@
       <c r="U23" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V23" s="2" t="n"/>
+      <c r="V23" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 1, Toán tăng cường 1</t>
+        </is>
+      </c>
+      <c r="W23" s="2" t="n"/>
     </row>
     <row r="24" ht="25" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -1942,7 +1853,12 @@
       <c r="U24" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V24" s="2" t="n"/>
+      <c r="V24" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 1, Toán tăng cường 1</t>
+        </is>
+      </c>
+      <c r="W24" s="2" t="n"/>
     </row>
     <row r="25" ht="25" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -1994,7 +1910,12 @@
       <c r="U25" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V25" s="2" t="n"/>
+      <c r="V25" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 1, Toán tăng cường 1</t>
+        </is>
+      </c>
+      <c r="W25" s="2" t="n"/>
     </row>
     <row r="26" ht="25" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -2046,7 +1967,12 @@
       <c r="U26" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V26" s="2" t="n"/>
+      <c r="V26" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 1, Toán tăng cường 1</t>
+        </is>
+      </c>
+      <c r="W26" s="2" t="n"/>
     </row>
     <row r="27" ht="25" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -2098,7 +2024,12 @@
       <c r="U27" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V27" s="2" t="n"/>
+      <c r="V27" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 1, Toán tăng cường 1</t>
+        </is>
+      </c>
+      <c r="W27" s="2" t="n"/>
     </row>
     <row r="28" ht="25" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -2150,7 +2081,12 @@
       <c r="U28" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V28" s="2" t="n"/>
+      <c r="V28" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 1, Toán tăng cường 1</t>
+        </is>
+      </c>
+      <c r="W28" s="2" t="n"/>
     </row>
     <row r="29" ht="25" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
@@ -2202,7 +2138,12 @@
       <c r="U29" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V29" s="2" t="n"/>
+      <c r="V29" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 1, Toán tăng cường 1</t>
+        </is>
+      </c>
+      <c r="W29" s="2" t="n"/>
     </row>
     <row r="30" ht="25" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -2252,7 +2193,12 @@
       <c r="U30" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V30" s="2" t="n"/>
+      <c r="V30" s="2" t="inlineStr">
+        <is>
+          <t>Tiếng Việt 2</t>
+        </is>
+      </c>
+      <c r="W30" s="2" t="n"/>
     </row>
     <row r="31" ht="25" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
@@ -2295,6 +2241,7 @@
       </c>
       <c r="U31" s="4" t="n"/>
       <c r="V31" s="4" t="n"/>
+      <c r="W31" s="4" t="n"/>
     </row>
     <row r="32" ht="25" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
@@ -2339,6 +2286,7 @@
       </c>
       <c r="U32" s="4" t="n"/>
       <c r="V32" s="4" t="n"/>
+      <c r="W32" s="4" t="n"/>
     </row>
     <row r="33" ht="25" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -2383,6 +2331,7 @@
       </c>
       <c r="U33" s="4" t="n"/>
       <c r="V33" s="4" t="n"/>
+      <c r="W33" s="4" t="n"/>
     </row>
     <row r="34" ht="25" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
@@ -2425,6 +2374,7 @@
       </c>
       <c r="U34" s="4" t="n"/>
       <c r="V34" s="4" t="n"/>
+      <c r="W34" s="4" t="n"/>
     </row>
     <row r="35" ht="25" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
@@ -2473,6 +2423,7 @@
       </c>
       <c r="U35" s="4" t="n"/>
       <c r="V35" s="4" t="n"/>
+      <c r="W35" s="4" t="n"/>
     </row>
     <row r="36" ht="25" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
@@ -2511,6 +2462,7 @@
       </c>
       <c r="U36" s="4" t="n"/>
       <c r="V36" s="4" t="n"/>
+      <c r="W36" s="4" t="n"/>
     </row>
     <row r="37" ht="25" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
@@ -2549,6 +2501,7 @@
       </c>
       <c r="U37" s="4" t="n"/>
       <c r="V37" s="4" t="n"/>
+      <c r="W37" s="4" t="n"/>
     </row>
     <row r="38" ht="25" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
@@ -2587,6 +2540,7 @@
       </c>
       <c r="U38" s="4" t="n"/>
       <c r="V38" s="4" t="n"/>
+      <c r="W38" s="4" t="n"/>
     </row>
     <row r="39" ht="25" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
@@ -2625,6 +2579,7 @@
       </c>
       <c r="U39" s="4" t="n"/>
       <c r="V39" s="4" t="n"/>
+      <c r="W39" s="4" t="n"/>
     </row>
     <row r="40" ht="25" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
@@ -2662,7 +2617,8 @@
         <v>23</v>
       </c>
       <c r="U40" s="5" t="n"/>
-      <c r="V40" s="5" t="n">
+      <c r="V40" s="5" t="n"/>
+      <c r="W40" s="5" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2702,7 +2658,8 @@
         <v>23</v>
       </c>
       <c r="U41" s="5" t="n"/>
-      <c r="V41" s="5" t="n">
+      <c r="V41" s="5" t="n"/>
+      <c r="W41" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2742,7 +2699,8 @@
         <v>23</v>
       </c>
       <c r="U42" s="5" t="n"/>
-      <c r="V42" s="5" t="n">
+      <c r="V42" s="5" t="n"/>
+      <c r="W42" s="5" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2783,6 +2741,7 @@
       </c>
       <c r="U43" s="4" t="n"/>
       <c r="V43" s="4" t="n"/>
+      <c r="W43" s="4" t="n"/>
     </row>
     <row r="44" ht="25" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
@@ -2821,6 +2780,7 @@
       </c>
       <c r="U44" s="4" t="n"/>
       <c r="V44" s="4" t="n"/>
+      <c r="W44" s="4" t="n"/>
     </row>
     <row r="45" ht="25" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
@@ -2858,7 +2818,8 @@
         <v>23</v>
       </c>
       <c r="U45" s="5" t="n"/>
-      <c r="V45" s="5" t="n">
+      <c r="V45" s="5" t="n"/>
+      <c r="W45" s="5" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2899,6 +2860,7 @@
       </c>
       <c r="U46" s="4" t="n"/>
       <c r="V46" s="4" t="n"/>
+      <c r="W46" s="4" t="n"/>
     </row>
     <row r="47" ht="25" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
@@ -2964,7 +2926,12 @@
       <c r="U47" s="1" t="n">
         <v>52</v>
       </c>
-      <c r="V47" s="1" t="n">
+      <c r="V47" s="1" t="inlineStr">
+        <is>
+          <t>39 ô</t>
+        </is>
+      </c>
+      <c r="W47" s="1" t="n">
         <v>17</v>
       </c>
     </row>
@@ -2981,7 +2948,7 @@
       <c r="A50" s="3" t="n"/>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>Môn có tiết dạy bù: 39 ô, 52 tiết (ghi chú trong ô ghi số tiết bù của môn)</t>
+          <t>Môn có tiết dạy bù: 39 ô, 52 tiết (số tiết từng môn ở cột Môn Dạy Bù)</t>
         </is>
       </c>
     </row>
@@ -2995,6 +2962,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Output template: statistics file with the sessions-off column
Regenerated with tools/mau_dau_ra.py (fake school, code 72C2-3315-CE24, same
timetable); only Output_Template_Thong_Ke_V8.xlsx changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B1DqxLw2MywB8g5N8E14F5
</commit_message>
<xml_diff>
--- a/data/Output_Template_Thong_Ke_V8.xlsx
+++ b/data/Output_Template_Thong_Ke_V8.xlsx
@@ -28,10 +28,12 @@
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
+      <color rgb="FF000000"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Times New Roman"/>
+      <color rgb="FF000000"/>
       <sz val="14"/>
     </font>
   </fonts>
@@ -464,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W51"/>
+  <dimension ref="A1:X51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20.3" customWidth="1" min="1" max="1"/>
@@ -490,6 +492,7 @@
     <col width="14.2" customWidth="1" min="21" max="21"/>
     <col width="39.7" customWidth="1" min="22" max="22"/>
     <col width="14.2" customWidth="1" min="23" max="23"/>
+    <col width="16.6" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -606,6 +609,11 @@
       <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Số Tiết Dư</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Số Buổi Nghỉ</t>
         </is>
       </c>
     </row>
@@ -659,6 +667,9 @@
         </is>
       </c>
       <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -710,6 +721,9 @@
         </is>
       </c>
       <c r="W3" s="2" t="n"/>
+      <c r="X3" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -761,6 +775,9 @@
         </is>
       </c>
       <c r="W4" s="2" t="n"/>
+      <c r="X4" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" ht="25" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -812,6 +829,9 @@
         </is>
       </c>
       <c r="W5" s="2" t="n"/>
+      <c r="X5" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" ht="25" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -863,6 +883,9 @@
         </is>
       </c>
       <c r="W6" s="2" t="n"/>
+      <c r="X6" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" ht="25" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -914,6 +937,9 @@
         </is>
       </c>
       <c r="W7" s="2" t="n"/>
+      <c r="X7" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" ht="25" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -967,6 +993,9 @@
         </is>
       </c>
       <c r="W8" s="2" t="n"/>
+      <c r="X8" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" ht="25" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -1020,6 +1049,9 @@
         </is>
       </c>
       <c r="W9" s="2" t="n"/>
+      <c r="X9" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" ht="25" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1073,6 +1105,9 @@
         </is>
       </c>
       <c r="W10" s="2" t="n"/>
+      <c r="X10" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" ht="25" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -1126,6 +1161,9 @@
         </is>
       </c>
       <c r="W11" s="2" t="n"/>
+      <c r="X11" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" ht="25" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1179,6 +1217,9 @@
         </is>
       </c>
       <c r="W12" s="2" t="n"/>
+      <c r="X12" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" ht="25" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -1232,6 +1273,9 @@
         </is>
       </c>
       <c r="W13" s="2" t="n"/>
+      <c r="X13" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" ht="25" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1289,6 +1333,9 @@
         </is>
       </c>
       <c r="W14" s="2" t="n"/>
+      <c r="X14" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" ht="25" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -1346,6 +1393,9 @@
         </is>
       </c>
       <c r="W15" s="2" t="n"/>
+      <c r="X15" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" ht="25" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -1403,6 +1453,9 @@
         </is>
       </c>
       <c r="W16" s="2" t="n"/>
+      <c r="X16" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" ht="25" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -1460,6 +1513,9 @@
         </is>
       </c>
       <c r="W17" s="2" t="n"/>
+      <c r="X17" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18" ht="25" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -1517,6 +1573,9 @@
         </is>
       </c>
       <c r="W18" s="2" t="n"/>
+      <c r="X18" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" ht="25" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -1574,6 +1633,9 @@
         </is>
       </c>
       <c r="W19" s="2" t="n"/>
+      <c r="X19" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" ht="25" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -1631,6 +1693,9 @@
         </is>
       </c>
       <c r="W20" s="2" t="n"/>
+      <c r="X20" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" ht="25" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -1688,6 +1753,9 @@
         </is>
       </c>
       <c r="W21" s="2" t="n"/>
+      <c r="X21" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22" ht="25" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -1745,6 +1813,9 @@
         </is>
       </c>
       <c r="W22" s="2" t="n"/>
+      <c r="X22" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23" ht="25" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -1802,6 +1873,9 @@
         </is>
       </c>
       <c r="W23" s="2" t="n"/>
+      <c r="X23" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24" ht="25" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -1859,6 +1933,9 @@
         </is>
       </c>
       <c r="W24" s="2" t="n"/>
+      <c r="X24" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25" ht="25" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -1916,6 +1993,9 @@
         </is>
       </c>
       <c r="W25" s="2" t="n"/>
+      <c r="X25" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26" ht="25" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -1973,6 +2053,9 @@
         </is>
       </c>
       <c r="W26" s="2" t="n"/>
+      <c r="X26" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27" ht="25" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -2030,6 +2113,9 @@
         </is>
       </c>
       <c r="W27" s="2" t="n"/>
+      <c r="X27" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" ht="25" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -2087,6 +2173,9 @@
         </is>
       </c>
       <c r="W28" s="2" t="n"/>
+      <c r="X28" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29" ht="25" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
@@ -2144,6 +2233,9 @@
         </is>
       </c>
       <c r="W29" s="2" t="n"/>
+      <c r="X29" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30" ht="25" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -2199,6 +2291,9 @@
         </is>
       </c>
       <c r="W30" s="2" t="n"/>
+      <c r="X30" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" ht="25" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
@@ -2242,6 +2337,9 @@
       <c r="U31" s="4" t="n"/>
       <c r="V31" s="4" t="n"/>
       <c r="W31" s="4" t="n"/>
+      <c r="X31" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32" ht="25" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
@@ -2287,6 +2385,9 @@
       <c r="U32" s="4" t="n"/>
       <c r="V32" s="4" t="n"/>
       <c r="W32" s="4" t="n"/>
+      <c r="X32" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33" ht="25" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -2332,6 +2433,9 @@
       <c r="U33" s="4" t="n"/>
       <c r="V33" s="4" t="n"/>
       <c r="W33" s="4" t="n"/>
+      <c r="X33" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34" ht="25" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
@@ -2375,6 +2479,9 @@
       <c r="U34" s="4" t="n"/>
       <c r="V34" s="4" t="n"/>
       <c r="W34" s="4" t="n"/>
+      <c r="X34" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35" ht="25" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
@@ -2424,6 +2531,9 @@
       <c r="U35" s="4" t="n"/>
       <c r="V35" s="4" t="n"/>
       <c r="W35" s="4" t="n"/>
+      <c r="X35" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36" ht="25" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
@@ -2463,6 +2573,9 @@
       <c r="U36" s="4" t="n"/>
       <c r="V36" s="4" t="n"/>
       <c r="W36" s="4" t="n"/>
+      <c r="X36" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37" ht="25" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
@@ -2502,6 +2615,9 @@
       <c r="U37" s="4" t="n"/>
       <c r="V37" s="4" t="n"/>
       <c r="W37" s="4" t="n"/>
+      <c r="X37" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38" ht="25" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
@@ -2541,6 +2657,9 @@
       <c r="U38" s="4" t="n"/>
       <c r="V38" s="4" t="n"/>
       <c r="W38" s="4" t="n"/>
+      <c r="X38" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39" ht="25" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
@@ -2580,6 +2699,9 @@
       <c r="U39" s="4" t="n"/>
       <c r="V39" s="4" t="n"/>
       <c r="W39" s="4" t="n"/>
+      <c r="X39" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40" ht="25" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
@@ -2621,6 +2743,9 @@
       <c r="W40" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="X40" s="5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="41" ht="25" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
@@ -2662,6 +2787,9 @@
       <c r="W41" s="5" t="n">
         <v>1</v>
       </c>
+      <c r="X41" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42" ht="25" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
@@ -2702,6 +2830,9 @@
       <c r="V42" s="5" t="n"/>
       <c r="W42" s="5" t="n">
         <v>5</v>
+      </c>
+      <c r="X42" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="43" ht="25" customHeight="1">
@@ -2742,6 +2873,9 @@
       <c r="U43" s="4" t="n"/>
       <c r="V43" s="4" t="n"/>
       <c r="W43" s="4" t="n"/>
+      <c r="X43" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44" ht="25" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
@@ -2781,6 +2915,9 @@
       <c r="U44" s="4" t="n"/>
       <c r="V44" s="4" t="n"/>
       <c r="W44" s="4" t="n"/>
+      <c r="X44" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45" ht="25" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
@@ -2822,6 +2959,9 @@
       <c r="W45" s="5" t="n">
         <v>6</v>
       </c>
+      <c r="X45" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46" ht="25" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
@@ -2861,6 +3001,9 @@
       <c r="U46" s="4" t="n"/>
       <c r="V46" s="4" t="n"/>
       <c r="W46" s="4" t="n"/>
+      <c r="X46" s="4" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="47" ht="25" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
@@ -2933,6 +3076,9 @@
       </c>
       <c r="W47" s="1" t="n">
         <v>17</v>
+      </c>
+      <c r="X47" s="1" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="48"/>

</xml_diff>

<commit_message>
Output templates: teacher timetable and quality sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VN2Svo1ahBQNvopmtaM579
</commit_message>
<xml_diff>
--- a/data/Output_Template_Thong_Ke_V8.xlsx
+++ b/data/Output_Template_Thong_Ke_V8.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Thống kê" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Chất lượng" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,10 +29,12 @@
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
+      <color rgb="FF000000"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Times New Roman"/>
+      <color rgb="FF000000"/>
       <sz val="14"/>
     </font>
   </fonts>
@@ -2963,4 +2966,648 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25.1" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="20.3" customWidth="1" min="3" max="3"/>
+    <col width="22.7" customWidth="1" min="4" max="4"/>
+    <col width="11.7" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nhóm</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Luật</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Mức</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Số Lần Không Theo</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Điểm Trừ</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Ví Dụ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="63" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Bảo vệ học sinh</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Mỗi buổi, một lớp học tối đa 2 tiết của một môn, tính chung môn chính với môn tăng cường cùng nhóm</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Bảo vệ học sinh</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Mỗi ngày, một lớp học tối đa 1 tiết Toán, khi số tiết/tuần của môn không quá số ngày học</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
+    </row>
+    <row r="4" ht="84" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Bảo vệ học sinh</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Môn có từ 6 tiết/tuần trở lên và số tiết chẵn, tính chung môn tăng cường cùng nhóm, học thành cặp 2 tiết liền trong buổi; trừ môn có nhãn Không ghép cặp</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Bảo vệ học sinh</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Các tiết của một môn trong cùng buổi phải đứng liền nhau</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Bảo vệ học sinh</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Trong một ngày, tiết môn tăng cường đứng sau các tiết môn chính cùng nhóm</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Bảo vệ học sinh</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Ngày có tiết môn tăng cường thì cũng có tiết môn chính cùng nhóm</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4" t="n"/>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>HĐTN và GVCN</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Ở mỗi giờ có nhãn Tiết HĐTN cố định, mỗi lớp học đúng 1 tiết HĐTN</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="4" t="n"/>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>HĐTN và GVCN</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Tiết HĐTN chỉ xếp vào giờ có nhãn Tiết HĐTN cố định hoặc Xếp tiết HĐTN còn lại</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4" t="n"/>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>HĐTN và GVCN</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Tiết HĐTN còn lại, ngoài giờ cố định, xếp ở tiết cuối buổi</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên thấp</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4" t="n"/>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>HĐTN và GVCN</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Ở giờ có nhãn Luôn do GVCN dạy, lớp học với GV chủ nhiệm</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>HĐTN và GVCN</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Môn có nhãn Chỉ GVCN dạy thì chỉ GV chủ nhiệm dạy</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="4" t="n"/>
+      <c r="F12" s="4" t="n"/>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Người dạy</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Hai tiết liền nhau của một môn (cùng nhóm) trong buổi do cùng một giáo viên dạy</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="4" t="n"/>
+      <c r="F13" s="4" t="n"/>
+    </row>
+    <row r="14" ht="63" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Người dạy</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Môn có nhãn GVCN nhận trọn: tiết đầu tuần của lớp do GV chủ nhiệm dạy, tiết của giáo viên khác không đứng trước</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Lịch giáo viên</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Giáo viên không dạy vào buổi nghỉ ghi ở cột Buổi Nghỉ và nghỉ đủ số buổi ghi ở đó</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n"/>
+      <c r="E15" s="4" t="n"/>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>kiểm bằng bộ kiểm tra độc lập</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="25" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Lịch giáo viên</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Mỗi buổi, một giáo viên chỉ dạy ở một cơ sở</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="n"/>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Lịch giáo viên</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Hạn chế để một giáo viên dạy ở cả hai cơ sở trong cùng một ngày</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên rất cao</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="4" t="n"/>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Lịch giáo viên</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Giáo viên không chủ nhiệm ghi Cơ sở 2 hoặc Thai Sản chỉ dạy các lớp ở cơ sở 2</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>kiểm bằng bộ kiểm tra độc lập</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="63" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên khi xếp giờ</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Tránh xếp môn có nhãn Môn nặng vào giờ có nhãn Hạn chế môn nặng</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên cao</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>4800</v>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>lớp 2/1 có Tiếng Anh Thứ 2 tiết 7; lớp 2/6 có Tiếng Anh Thứ 2 tiết 7; lớp 4/5 có Tiếng Anh Thứ 2 tiết 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="63" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên khi xếp giờ</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Môn có nhãn Ưu tiên buổi sáng xếp vào buổi sáng</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên vừa</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>10800</v>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>lớp 1/1 có Tiếng Việt Thứ 4 tiết 5; lớp 1/1 có Tiếng Việt Thứ 4 tiết 6; lớp 1/2 có Tiếng Việt Thứ 4 tiết 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="63" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên khi xếp giờ</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Số tiết mỗi ngày của giáo viên không quá tải ngày, tức số tiết/tuần chia đều cho các ngày</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên thấp</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Bộ Môn 1 Thứ 4: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 1 Thứ 5: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 2 Thứ 3: 6 tiết (tối đa 5 = tải ngày)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="84" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên khi xếp giờ</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Số tiết mỗi ngày của giáo viên không quá tải ngày + 1 tiết</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên vừa</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>2700</v>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Chủ Nhiệm 1/3 Thứ 5: 6 tiết (tối đa 5 = tải ngày + 1); Chủ Nhiệm 1/5 Thứ 3: 6 tiết (tối đa 5 = tải ngày + 1); Chủ Nhiệm 1/6 Thứ 3: 6 tiết (tối đa 5 = tải ngày + 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="105" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên khi xếp giờ</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Mỗi môn, trừ HĐTN và môn ưu tiên buổi sáng, rải đều trong tuần: một ngày không quá số tiết/tuần chia số ngày</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên thấp</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>280</v>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>lớp 1/5 Tiếng Anh Thứ 6: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/1 Tiếng Việt tăng cường Thứ 2: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/2 Tiếng Việt tăng cường Thứ 3: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="105" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên khi xếp giờ</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Môn ưu tiên buổi sáng rải đều trong tuần: một ngày không quá số tiết/tuần chia số ngày</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên thấp</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>1560</v>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>lớp 1/1 Tiếng Việt Thứ 4: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/1 Tiếng Việt Thứ 5: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/2 Tiếng Việt Thứ 4: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên khi xếp giờ</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Giáo viên, trừ GV chủ nhiệm, không có tiết trống xen giữa các tiết trong buổi</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên thấp</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="4" t="n"/>
+    </row>
+    <row r="26" ht="25" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>Tổng</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="n"/>
+      <c r="C26" s="1" t="n"/>
+      <c r="D26" s="1" t="n">
+        <v>149</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>28140</v>
+      </c>
+      <c r="F26" s="1" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update reference codes, output templates and docs for the overtime fix
Linux codes after the fix: small school 5444-2BE7-93B3 / 1F0E-EA75-72A3,
school file FF2F-F451-28ED, fake school 515A-B49D-D6A7. The quality sheet
now matches the solver cost (fake school 25,140; school file quality
39,120 -> 34,780 points at the same budget). Windows codes follow from CI.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WtuWVKdziZbvQ9VXgRdGv
</commit_message>
<xml_diff>
--- a/data/Output_Template_Thong_Ke_V8.xlsx
+++ b/data/Output_Template_Thong_Ke_V8.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Thống kê" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Chất lượng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thống kê" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chất lượng" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3423,7 +3423,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>lớp 2/1 có Tiếng Anh Thứ 2 tiết 7; lớp 2/6 có Tiếng Anh Thứ 2 tiết 7; lớp 4/5 có Tiếng Anh Thứ 2 tiết 7</t>
+          <t>lớp 2/3 có Tiếng Anh Thứ 2 tiết 7; lớp 2/6 có Tiếng Anh Thứ 2 tiết 7; lớp 3/6 có Tiếng Anh Thứ 4 tiết 7</t>
         </is>
       </c>
     </row>
@@ -3444,14 +3444,14 @@
         </is>
       </c>
       <c r="D20" s="4" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>10800</v>
+        <v>11100</v>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>lớp 1/1 có Tiếng Việt Thứ 4 tiết 5; lớp 1/1 có Tiếng Việt Thứ 4 tiết 6; lớp 1/2 có Tiếng Việt Thứ 4 tiết 5</t>
+          <t>lớp 1/1 có Tiếng Việt Thứ 2 tiết 5; lớp 1/1 có Tiếng Việt Thứ 2 tiết 6; lớp 1/1 có Tiếng Việt Thứ 4 tiết 5</t>
         </is>
       </c>
     </row>
@@ -3472,18 +3472,18 @@
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>8000</v>
+        <v>7100</v>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Bộ Môn 1 Thứ 4: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 1 Thứ 5: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 2 Thứ 3: 6 tiết (tối đa 5 = tải ngày)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="84" customHeight="1">
+          <t>Bộ Môn 1 Thứ 5: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 2 Thứ 3: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 3 Thứ 4: 6 tiết (tối đa 5 = tải ngày)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="42" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Ưu tiên khi xếp giờ</t>
@@ -3500,14 +3500,14 @@
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>2700</v>
+        <v>300</v>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Chủ Nhiệm 1/3 Thứ 5: 6 tiết (tối đa 5 = tải ngày + 1); Chủ Nhiệm 1/5 Thứ 3: 6 tiết (tối đa 5 = tải ngày + 1); Chủ Nhiệm 1/6 Thứ 3: 6 tiết (tối đa 5 = tải ngày + 1)</t>
+          <t>Chủ Nhiệm 1/2 Thứ 2: 6 tiết (tối đa 5 = tải ngày + 1)</t>
         </is>
       </c>
     </row>
@@ -3535,7 +3535,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>lớp 1/5 Tiếng Anh Thứ 6: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/1 Tiếng Việt tăng cường Thứ 2: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/2 Tiếng Việt tăng cường Thứ 3: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày)</t>
+          <t>lớp 1/2 Tiếng Anh Thứ 6: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/1 Tiếng Việt tăng cường Thứ 4: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/2 Tiếng Việt tăng cường Thứ 3: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày)</t>
         </is>
       </c>
     </row>
@@ -3563,7 +3563,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>lớp 1/1 Tiếng Việt Thứ 4: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/1 Tiếng Việt Thứ 5: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/2 Tiếng Việt Thứ 4: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày)</t>
+          <t>lớp 1/1 Tiếng Việt Thứ 4: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/1 Tiếng Việt Thứ 5: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/2 Tiếng Việt Thứ 2: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày)</t>
         </is>
       </c>
     </row>
@@ -3600,10 +3600,10 @@
       <c r="B26" s="1" t="n"/>
       <c r="C26" s="1" t="n"/>
       <c r="D26" s="1" t="n">
-        <v>149</v>
+        <v>133</v>
       </c>
       <c r="E26" s="1" t="n">
-        <v>28140</v>
+        <v>25140</v>
       </c>
       <c r="F26" s="1" t="n"/>
     </row>

</xml_diff>

<commit_message>
Regenerate output templates and record the new sample results
The fake school now gives 187E-B6C1-A93B on Linux (24 740 points,
was 25 140). Spec: history row 83 and the section 13 sample numbers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WtuWVKdziZbvQ9VXgRdGv
</commit_message>
<xml_diff>
--- a/data/Output_Template_Thong_Ke_V8.xlsx
+++ b/data/Output_Template_Thong_Ke_V8.xlsx
@@ -3359,7 +3359,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Hạn chế để một giáo viên dạy ở cả hai cơ sở trong cùng một ngày</t>
+          <t>Hạn chế để một giáo viên đổi cơ sở trong cùng một ngày (dạy ở hai cơ sở trở lên)</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>lớp 2/3 có Tiếng Anh Thứ 2 tiết 7; lớp 2/6 có Tiếng Anh Thứ 2 tiết 7; lớp 3/6 có Tiếng Anh Thứ 4 tiết 7</t>
+          <t>lớp 1/4 có Tiếng Anh Thứ 2 tiết 7; lớp 3/4 có Tiếng Anh Thứ 4 tiết 7; lớp 4/2 có Tiếng Anh Thứ 2 tiết 7</t>
         </is>
       </c>
     </row>
@@ -3444,14 +3444,14 @@
         </is>
       </c>
       <c r="D20" s="4" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>11100</v>
+        <v>10800</v>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>lớp 1/1 có Tiếng Việt Thứ 2 tiết 5; lớp 1/1 có Tiếng Việt Thứ 2 tiết 6; lớp 1/1 có Tiếng Việt Thứ 4 tiết 5</t>
+          <t>lớp 1/1 có Tiếng Việt Thứ 3 tiết 5; lớp 1/1 có Tiếng Việt Thứ 3 tiết 6; lớp 1/1 có Tiếng Việt Thứ 4 tiết 5</t>
         </is>
       </c>
     </row>
@@ -3472,14 +3472,14 @@
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>7100</v>
+        <v>7300</v>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Bộ Môn 1 Thứ 5: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 2 Thứ 3: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 3 Thứ 4: 6 tiết (tối đa 5 = tải ngày)</t>
+          <t>Bộ Môn 1 Thứ 4: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 1 Thứ 5: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 2 Thứ 3: 6 tiết (tối đa 5 = tải ngày)</t>
         </is>
       </c>
     </row>
@@ -3500,16 +3500,12 @@
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>300</v>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Chủ Nhiệm 1/2 Thứ 2: 6 tiết (tối đa 5 = tải ngày + 1)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F22" s="4" t="n"/>
     </row>
     <row r="23" ht="105" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
@@ -3535,7 +3531,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>lớp 1/2 Tiếng Anh Thứ 6: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/1 Tiếng Việt tăng cường Thứ 4: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/2 Tiếng Việt tăng cường Thứ 3: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày)</t>
+          <t>lớp 1/5 Tiếng Anh Thứ 6: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/1 Tiếng Việt tăng cường Thứ 3: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/2 Tiếng Việt tăng cường Thứ 4: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày)</t>
         </is>
       </c>
     </row>
@@ -3563,7 +3559,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>lớp 1/1 Tiếng Việt Thứ 4: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/1 Tiếng Việt Thứ 5: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/2 Tiếng Việt Thứ 2: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày)</t>
+          <t>lớp 1/1 Tiếng Việt Thứ 3: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/1 Tiếng Việt Thứ 4: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/2 Tiếng Việt Thứ 3: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày)</t>
         </is>
       </c>
     </row>
@@ -3603,7 +3599,7 @@
         <v>133</v>
       </c>
       <c r="E26" s="1" t="n">
-        <v>25140</v>
+        <v>24740</v>
       </c>
       <c r="F26" s="1" t="n"/>
     </row>

</xml_diff>

<commit_message>
Record the Linux codes after the hot spot change
main.py on the school file gives 73BC-265B-29F2 on Linux (34 300
points, no campus change), the fake school 4DCC-D5FC-F768 (24 860).
Output templates regenerated. Windows codes follow from CI.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WtuWVKdziZbvQ9VXgRdGv
</commit_message>
<xml_diff>
--- a/data/Output_Template_Thong_Ke_V8.xlsx
+++ b/data/Output_Template_Thong_Ke_V8.xlsx
@@ -3423,7 +3423,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>lớp 1/4 có Tiếng Anh Thứ 2 tiết 7; lớp 3/4 có Tiếng Anh Thứ 4 tiết 7; lớp 4/2 có Tiếng Anh Thứ 2 tiết 7</t>
+          <t>lớp 1/6 có Tiếng Anh Thứ 2 tiết 7; lớp 3/3 có Tiếng Anh Thứ 2 tiết 7; lớp 4/3 có Tiếng Anh Thứ 5 tiết 7</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>lớp 1/1 có Tiếng Việt Thứ 3 tiết 5; lớp 1/1 có Tiếng Việt Thứ 3 tiết 6; lớp 1/1 có Tiếng Việt Thứ 4 tiết 5</t>
+          <t>lớp 1/1 có Tiếng Việt Thứ 3 tiết 5; lớp 1/1 có Tiếng Việt Thứ 3 tiết 6; lớp 1/1 có Tiếng Việt Thứ 5 tiết 5</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Bộ Môn 1 Thứ 4: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 1 Thứ 5: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 2 Thứ 3: 6 tiết (tối đa 5 = tải ngày)</t>
+          <t>Bộ Môn 1 Thứ 5: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 2 Thứ 4: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 2 Thứ 5: 6 tiết (tối đa 5 = tải ngày)</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>lớp 1/5 Tiếng Anh Thứ 6: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/1 Tiếng Việt tăng cường Thứ 3: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/2 Tiếng Việt tăng cường Thứ 4: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày)</t>
+          <t>lớp 2/1 Tiếng Anh Thứ 6: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/1 Tiếng Việt tăng cường Thứ 3: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/2 Tiếng Việt tăng cường Thứ 4: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày)</t>
         </is>
       </c>
     </row>
@@ -3552,14 +3552,14 @@
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>1560</v>
+        <v>1680</v>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>lớp 1/1 Tiếng Việt Thứ 3: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/1 Tiếng Việt Thứ 4: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/2 Tiếng Việt Thứ 3: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày)</t>
+          <t>lớp 1/1 Tiếng Việt Thứ 3: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/1 Tiếng Việt Thứ 5: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/2 Tiếng Việt Thứ 4: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày)</t>
         </is>
       </c>
     </row>
@@ -3596,10 +3596,10 @@
       <c r="B26" s="1" t="n"/>
       <c r="C26" s="1" t="n"/>
       <c r="D26" s="1" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E26" s="1" t="n">
-        <v>24740</v>
+        <v>24860</v>
       </c>
       <c r="F26" s="1" t="n"/>
     </row>

</xml_diff>

<commit_message>
Regenerate output templates and fake-school results for the faster LNS
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WtuWVKdziZbvQ9VXgRdGv
</commit_message>
<xml_diff>
--- a/data/Output_Template_Thong_Ke_V8.xlsx
+++ b/data/Output_Template_Thong_Ke_V8.xlsx
@@ -3423,7 +3423,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>lớp 1/6 có Tiếng Anh Thứ 2 tiết 7; lớp 3/3 có Tiếng Anh Thứ 2 tiết 7; lớp 4/3 có Tiếng Anh Thứ 5 tiết 7</t>
+          <t>lớp 1/3 có Tiếng Anh Thứ 2 tiết 7; lớp 2/6 có Tiếng Anh Thứ 2 tiết 7; lớp 4/2 có Tiếng Anh Thứ 4 tiết 7</t>
         </is>
       </c>
     </row>
@@ -3444,14 +3444,14 @@
         </is>
       </c>
       <c r="D20" s="4" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>10800</v>
+        <v>11100</v>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>lớp 1/1 có Tiếng Việt Thứ 3 tiết 5; lớp 1/1 có Tiếng Việt Thứ 3 tiết 6; lớp 1/1 có Tiếng Việt Thứ 5 tiết 5</t>
+          <t>lớp 1/1 có Tiếng Việt Thứ 3 tiết 5; lớp 1/1 có Tiếng Việt Thứ 3 tiết 6; lớp 1/1 có Tiếng Việt Thứ 4 tiết 5</t>
         </is>
       </c>
     </row>
@@ -3472,14 +3472,14 @@
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>7300</v>
+        <v>7100</v>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Bộ Môn 1 Thứ 5: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 2 Thứ 4: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 2 Thứ 5: 6 tiết (tối đa 5 = tải ngày)</t>
+          <t>Bộ Môn 1 Thứ 5: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 2 Thứ 5: 6 tiết (tối đa 5 = tải ngày); Bộ Môn 3 Thứ 3: 6 tiết (tối đa 5 = tải ngày)</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>lớp 2/1 Tiếng Anh Thứ 6: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/1 Tiếng Việt tăng cường Thứ 3: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/2 Tiếng Việt tăng cường Thứ 4: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày)</t>
+          <t>lớp 2/1 Tiếng Anh Thứ 6: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/1 Tiếng Việt tăng cường Thứ 3: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày); lớp 2/2 Tiếng Việt tăng cường Thứ 5: 2 tiết (tối đa 1 = số tiết/tuần chia số ngày)</t>
         </is>
       </c>
     </row>
@@ -3559,7 +3559,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>lớp 1/1 Tiếng Việt Thứ 3: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/1 Tiếng Việt Thứ 5: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/2 Tiếng Việt Thứ 4: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày)</t>
+          <t>lớp 1/1 Tiếng Việt Thứ 3: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/1 Tiếng Việt Thứ 4: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày); lớp 1/2 Tiếng Việt Thứ 4: 4 tiết (tối đa 3 = số tiết/tuần chia số ngày)</t>
         </is>
       </c>
     </row>
@@ -3596,10 +3596,10 @@
       <c r="B26" s="1" t="n"/>
       <c r="C26" s="1" t="n"/>
       <c r="D26" s="1" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E26" s="1" t="n">
-        <v>24860</v>
+        <v>24960</v>
       </c>
       <c r="F26" s="1" t="n"/>
     </row>

</xml_diff>